<commit_message>
Screening check: blinded reading of 50 records and its scores
</commit_message>
<xml_diff>
--- a/data/deposit/R01_screening_workbook.xlsx
+++ b/data/deposit/R01_screening_workbook.xlsx
@@ -80204,7 +80204,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -80213,7 +80213,131 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>The blinded check sample has not been scored yet (pipeline/03_check_screening.py sample, then score).</t>
+          <t>Screening check: 50 records read blind to the rules' decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Confusion matrix (rows: reader, columns: rules)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>rules_decision   Include  Maybe  Exclude</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">reader_decision                         </t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Include               19      4        1</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Maybe                  0      7        2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Exclude                1      4       12</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Rules Include: reader agreed on 19 of 20</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Rules Maybe: reader agreed on 7 of 15</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Rules Exclude: reader agreed on 12 of 15</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Estimates for all 1059 screened records (stratum-weighted):</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  recall (rules do not exclude a reader-Include record): 0.997 (95% CI 0.990 to 1.000)  -&gt; meets the pre-specified threshold 0.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  strict recall (rules Include):                        0.993 (95% CI 0.985 to 0.998)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  specificity (rules Exclude a reader-Exclude record):   0.395 (95% CI 0.167 to 0.957)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  agreement, three classes:                              0.937 (95% CI 0.837 to 0.991)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  eligible records among the 44 the rules exclude: 2.9 (95% CI 0.0 to 8.8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>On the sample: agreement 0.760; Cohen's kappa 0.632 (95% CI 0.472 to 0.787); PABAK 0.640 (95% CI 0.490 to 0.790)</t>
         </is>
       </c>
     </row>

</xml_diff>